<commit_message>
Gerados arquivos de otimização
</commit_message>
<xml_diff>
--- a/Fazenda Campo Dourado/ingredientes_racoes_GO_campo_dourado.xlsx
+++ b/Fazenda Campo Dourado/ingredientes_racoes_GO_campo_dourado.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -110,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -142,6 +143,16 @@
     <xf numFmtId="164" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -519,6 +530,10 @@
     <col width="11" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="95" customWidth="1" min="12" max="12"/>
+    <col width="75" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -576,6 +591,27 @@
 ( purchased_feed_cost )</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Preço
+(R$/t matéria natural)</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Preço original</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Fonte do preço</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Conversão / observação</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="n">
@@ -606,8 +642,26 @@
       <c r="H4" s="6" t="n">
         <v>0.195</v>
       </c>
-      <c r="I4" s="5" t="n">
-        <v>0.01</v>
+      <c r="I4" s="11" t="n">
+        <v>1.8207</v>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>1700</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>R$ 1,70/kg (fardo 15–17 kg)</t>
+        </is>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>MF Rural – anúncio "Feno Tifton e Jiggs – Fardo", Campo Verde/MT (acesso 28/10/2026) – https://www.mfrural.com.br/busca/feno-tifton</t>
+        </is>
+      </c>
+      <c r="M4" s="13" t="inlineStr">
+        <is>
+          <t>Tifton 85 é Cynodon (bermudagrass). Anúncio mais próximo de GO com preço por kg. 1.7000 R$/kg MN ÷ 0.9337 MS = 1.8207 R$/kg MS</t>
+        </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -639,8 +693,28 @@
       <c r="H5" s="10" t="n">
         <v>0.276</v>
       </c>
-      <c r="I5" s="9" t="n">
-        <v>0.1</v>
+      <c r="I5" s="12" t="n">
+        <v>999</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>Sem preço: uso proibido na alimentação de ruminantes no Brasil – IN MAPA nº 8/2004 – https://www.normasbrasil.com.br/norma/instrucao-normativa-8-2004_75298.html</t>
+        </is>
+      </c>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>Custo-penalidade 999 R$/kg MS para excluir o ingrediente do PL</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -672,8 +746,26 @@
       <c r="H6" s="6" t="n">
         <v>0.309</v>
       </c>
-      <c r="I6" s="5" t="n">
-        <v>0.5</v>
+      <c r="I6" s="11" t="n">
+        <v>1.2413</v>
+      </c>
+      <c r="J6" s="14" t="n">
+        <v>1078.83</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>R$ 64,73/saca 60 kg</t>
+        </is>
+      </c>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>CEPEA – Indicador do Milho ESALQ/BM&amp;FBOVESPA, 28/10/2026 – https://www.cepea.org.br/br/indicador/milho.aspx</t>
+        </is>
+      </c>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t>64,73 ÷ 60 = 1,0788 R$/kg MN. 1.0788 R$/kg MN ÷ 0.8691 MS = 1.2413 R$/kg MS</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -705,8 +797,26 @@
       <c r="H7" s="10" t="n">
         <v>0.232</v>
       </c>
-      <c r="I7" s="9" t="n">
-        <v>0.01</v>
+      <c r="I7" s="12" t="n">
+        <v>0.6988</v>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>247.08</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>R$ 247,08/t (custo de produção)</t>
+        </is>
+      </c>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>CNA/Senar + Cepea-Esalq – Ativos do Campo Pecuária de Leite, set/2026 (Projeto Campo Futuro, safra 25/26) – https://cnabrasil.org.br/storage/arquivos/files/Ativos-do-Campo-Pecuaria-de-Leite-Setembro2026.pdf</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>Custo médio de produção própria, 1ª safra, 18 propriedades típicas. 0.2471 R$/kg MN ÷ 0.3536 MS = 0.6988 R$/kg MS</t>
+        </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -738,8 +848,26 @@
       <c r="H8" s="6" t="n">
         <v>0.329</v>
       </c>
-      <c r="I8" s="5" t="n">
-        <v>0.01</v>
+      <c r="I8" s="11" t="n">
+        <v>2.5213</v>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>2250</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Tifton R$ 1,70/kg; alfafa R$ 2,80/kg</t>
+        </is>
+      </c>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>MF Rural – "Feno Tifton e Jiggs", Campo Verde/MT (https://www.mfrural.com.br/busca/feno-tifton) e "Alfafa Premium 20kg", São Luiz Gonzaga/RS (https://www.mfrural.com.br/busca/alfafa-fardo), acesso 28/10/2026</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>Estimativa: média 50/50 feno de capim + feno de leguminosa = 2,25 R$/kg MN. 2.2500 R$/kg MN ÷ 0.8924 MS = 2.5213 R$/kg MS</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -771,8 +899,26 @@
       <c r="H9" s="10" t="n">
         <v>0.341</v>
       </c>
-      <c r="I9" s="9" t="n">
-        <v>0.01</v>
+      <c r="I9" s="12" t="n">
+        <v>2.7486</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>1100</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>R$ 1,10/kg</t>
+        </is>
+      </c>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>MF Rural – "Feno Tifton 85 Pré-Secado", Luziânia/GO (acesso 28/10/2026) – https://www.mfrural.com.br/busca/pre-secado</t>
+        </is>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>Proxy: pré-secado (silagem pré-emurchecida) de Goiás. 1.1000 R$/kg MN ÷ 0.4002 MS = 2.7486 R$/kg MS</t>
+        </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -804,8 +950,26 @@
       <c r="H10" s="6" t="n">
         <v>0.351</v>
       </c>
-      <c r="I10" s="5" t="n">
-        <v>0.01</v>
+      <c r="I10" s="11" t="n">
+        <v>2.5653</v>
+      </c>
+      <c r="J10" s="14" t="n">
+        <v>1100</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>R$ 1,10/kg</t>
+        </is>
+      </c>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>MF Rural – "Feno Tifton 85 Pré-Secado", Luziânia/GO (acesso 28/10/2026) – https://www.mfrural.com.br/busca/pre-secado</t>
+        </is>
+      </c>
+      <c r="M10" s="13" t="inlineStr">
+        <is>
+          <t>Proxy: não há cotação de silagem de leguminosa; usado o pré-secado de GO (provavelmente subestima). 1.1000 R$/kg MN ÷ 0.4288 MS = 2.5653 R$/kg MS</t>
+        </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -837,8 +1001,26 @@
       <c r="H11" s="10" t="n">
         <v>0.266</v>
       </c>
-      <c r="I11" s="9" t="n">
-        <v>0.1</v>
+      <c r="I11" s="12" t="n">
+        <v>0.7851</v>
+      </c>
+      <c r="J11" s="14" t="n">
+        <v>247.08</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>R$ 247,08/t (custo silagem de milho)</t>
+        </is>
+      </c>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>CNA/Senar + Cepea-Esalq – Ativos do Campo Pecuária de Leite, set/2026 – https://cnabrasil.org.br/storage/arquivos/files/Ativos-do-Campo-Pecuaria-de-Leite-Setembro2026.pdf</t>
+        </is>
+      </c>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>Proxy: custo/t de silagem de sorgo ≈ milho (Embrapa Milho e Sorgo, Comparação de custos – https://www.alice.cnptia.embrapa.br/alice/bitstream/doc/472848/1/Comparacaocustos.pdf). 0.2471 R$/kg MN ÷ 0.3147 MS = 0.7851 R$/kg MS</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
@@ -870,8 +1052,26 @@
       <c r="H12" s="6" t="n">
         <v>0.75</v>
       </c>
-      <c r="I12" s="5" t="n">
-        <v>0.1</v>
+      <c r="I12" s="11" t="n">
+        <v>23.0171</v>
+      </c>
+      <c r="J12" s="14" t="n">
+        <v>2877.13</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>R$ 2,9692/litro</t>
+        </is>
+      </c>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t>CEPEA – Preço do leite ao produtor, Goiás, ago/2026 – https://www.cepea.org.br/br/indicador/leite.aspx</t>
+        </is>
+      </c>
+      <c r="M12" s="13" t="inlineStr">
+        <is>
+          <t>÷ 1,032 kg/L (densidade) = 2,8771 R$/kg MN; custo de oportunidade do leite. 2.8771 R$/kg MN ÷ 0.1250 MS = 23.0171 R$/kg MS</t>
+        </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -903,8 +1103,26 @@
       <c r="H13" s="10" t="n">
         <v>0.37</v>
       </c>
-      <c r="I13" s="9" t="n">
-        <v>0.1</v>
+      <c r="I13" s="12" t="n">
+        <v>2.856</v>
+      </c>
+      <c r="J13" s="14" t="n">
+        <v>2513.25</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>R$ 100,53/saco 40 kg</t>
+        </is>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>Loja Cocamar – "Ração para Bezerro 20%" (acesso 28/10/2026) – https://www.lojacocamar.com.br/racao-para-bezerro-20/p</t>
+        </is>
+      </c>
+      <c r="M13" s="13" t="inlineStr">
+        <is>
+          <t>100,53 ÷ 40 = 2,5133 R$/kg MN; produto indisponível no site no momento da consulta. 2.5133 R$/kg MN ÷ 0.8800 MS = 2.8560 R$/kg MS</t>
+        </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -936,8 +1154,26 @@
       <c r="H14" s="6" t="n">
         <v>2.32</v>
       </c>
-      <c r="I14" s="5" t="n">
-        <v>1</v>
+      <c r="I14" s="11" t="n">
+        <v>12.2904</v>
+      </c>
+      <c r="J14" s="14" t="n">
+        <v>12224</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>R$ 305,60/saco 25 kg</t>
+        </is>
+      </c>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>UFMA – Pregão nº 90032/2025 (jan/2026), Termo de Referência, item mineral p/ vacas em lactação – https://portalpadrao.ufma.br/ppgt/editais/05-01-2026-pregao-ndeg-90032-2025/tr154041_000141_2025.pdf</t>
+        </is>
+      </c>
+      <c r="M14" s="13" t="inlineStr">
+        <is>
+          <t>305,60 ÷ 25 = 12,224 R$/kg MN; preço de compra pública. 12.2240 R$/kg MN ÷ 0.9946 MS = 12.2904 R$/kg MS</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -946,12 +1182,12 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Premix mineral/vitamínico</t>
+          <t>Blend de subprodutos (concentrado proteico)</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Mineral</t>
+          <t>Concentrado proteico</t>
         </is>
       </c>
       <c r="D15" s="9" t="n">
@@ -969,8 +1205,26 @@
       <c r="H15" s="10" t="n">
         <v>0.73</v>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0.1</v>
+      <c r="I15" s="12" t="n">
+        <v>1.2159</v>
+      </c>
+      <c r="J15" s="14" t="n">
+        <v>901.11</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>DDGS de milho 28–36% PB: R$ 1.070/t (mediana de 11 anúncios a granel)</t>
+        </is>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>MF Rural – busca "DDG" (anúncios de MT, MS e SP, acesso 28/10/2026) – https://www.mfrural.com.br/busca/ddg ; MS do DDGS = 88% (Embrapa Suínos e Aves, Comunicado Técnico 594) – https://www.infoteca.cnptia.embrapa.br/infoteca/bitstream/doc/1149447/1/final10026.pdf</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t>Proxy: no NASEM_Comp o 303 é "Farm ES Northeast BP Blend" (Conc, 33% PB, 78% PNDR); DDGS é o subproduto proteico equivalente produzido em GO/MT. 1.070 R$/t ÷ 0,88 MS = 1.2159 R$/kg MS; × 0,7411 (MS do 303) = 901.11 R$/t MN. Preços FOB em MT/MS/SP, sem frete até GO</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>